<commit_message>
fixed ranks with week vs list
</commit_message>
<xml_diff>
--- a/007/ranks.xlsx
+++ b/007/ranks.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="117">
   <si>
     <t xml:space="preserve">Sparwoche</t>
   </si>
@@ -76,25 +76,31 @@
     <t xml:space="preserve">Fran171526</t>
   </si>
   <si>
+    <t xml:space="preserve">RAV28</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fürst der Nazgúl</t>
   </si>
   <si>
     <t xml:space="preserve">R4</t>
   </si>
   <si>
-    <t xml:space="preserve">RAV28</t>
-  </si>
-  <si>
     <t xml:space="preserve">SNEAKY BUNNY</t>
   </si>
   <si>
     <t xml:space="preserve">MrSajmonn</t>
   </si>
   <si>
+    <t xml:space="preserve">Bugab0o</t>
+  </si>
+  <si>
     <t xml:space="preserve">cappu97</t>
   </si>
   <si>
-    <t xml:space="preserve">Bugab0o</t>
+    <t xml:space="preserve">supi pupi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lefueT</t>
   </si>
   <si>
     <t xml:space="preserve">Bogo und Pini</t>
@@ -103,277 +109,271 @@
     <t xml:space="preserve">Haulsen</t>
   </si>
   <si>
-    <t xml:space="preserve">lefueT</t>
-  </si>
-  <si>
     <t xml:space="preserve">Jacob Carter</t>
   </si>
   <si>
+    <t xml:space="preserve">Gordon Freimann</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kytrider</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Smowy</t>
+  </si>
+  <si>
     <t xml:space="preserve">SmartesGirl</t>
   </si>
   <si>
+    <t xml:space="preserve">JSheridan</t>
+  </si>
+  <si>
     <t xml:space="preserve">Peridakles</t>
   </si>
   <si>
-    <t xml:space="preserve">supi pupi</t>
+    <t xml:space="preserve">Giorgiotown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SNPOL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marshalfey</t>
   </si>
   <si>
     <t xml:space="preserve">jobcenter FFM</t>
   </si>
   <si>
-    <t xml:space="preserve">Gordon Freimann</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marshalfey</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JSheridan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kytrider</t>
+    <t xml:space="preserve">Jónny666</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feivel D Maus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sugarpüff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K E R S Y</t>
   </si>
   <si>
     <t xml:space="preserve">2 s t y</t>
   </si>
   <si>
-    <t xml:space="preserve">Sugarpüff</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Smowy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Feivel D Maus</t>
-  </si>
-  <si>
     <t xml:space="preserve">Queen from AZO</t>
   </si>
   <si>
     <t xml:space="preserve">R5</t>
   </si>
   <si>
-    <t xml:space="preserve">K E R S Y</t>
-  </si>
-  <si>
     <t xml:space="preserve">DragonWiz</t>
   </si>
   <si>
-    <t xml:space="preserve">Jónny666</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SNPOL</t>
-  </si>
-  <si>
     <t xml:space="preserve">Himbeertony</t>
   </si>
   <si>
+    <t xml:space="preserve">Cluster82</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N</t>
+  </si>
+  <si>
     <t xml:space="preserve">ozzy5255</t>
   </si>
   <si>
     <t xml:space="preserve">Dejweed</t>
   </si>
   <si>
-    <t xml:space="preserve">N</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Giorgiotown</t>
+    <t xml:space="preserve">PHOENIX FOX</t>
   </si>
   <si>
     <t xml:space="preserve">Tom12234455</t>
   </si>
   <si>
-    <t xml:space="preserve">Cluster82</t>
+    <t xml:space="preserve">Svela17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CalziferFire</t>
   </si>
   <si>
     <t xml:space="preserve">fffeyz</t>
   </si>
   <si>
-    <t xml:space="preserve">CalziferFire</t>
+    <t xml:space="preserve">Hhjjjjcg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aenwe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Swe Sandman</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DaliborDaki</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feimel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CërëalKillër</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fürstin Elora</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Schlabberbacke</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tyskie 66</t>
+  </si>
+  <si>
+    <t xml:space="preserve">haasenpeter rex</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skywölkchen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sphere8472</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MetauChopf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dragon blou</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MiepStreet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sunny75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dr Cal Lightman</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lilien1999</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pawelte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xambash</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MG Mayo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last Arti</t>
+  </si>
+  <si>
+    <t xml:space="preserve">케포 부인</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cheesynator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">azerty57</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Katerina77</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EXITUS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sultan Murat X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kpiftw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Christo30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last Wolf Warrior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jukata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LatastrophenUlli</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Z4ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jimi777</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sanya Longer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mel Lyn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ECSI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yama Arashi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mischel89</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pinsel20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mac1902</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bestia77</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kurdo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GaaGol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DooYooDoo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leijonamieli</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FATUUM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Pharo 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toby Urbex</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VxClicker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yyyyyyyvhhmll</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R2DrehZwo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Points</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Li La Linus</t>
   </si>
   <si>
     <t xml:space="preserve">SamoZlo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CërëalKillër</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Swe Sandman</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DaliborDaki</t>
-  </si>
-  <si>
-    <t xml:space="preserve">feimel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aenwe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PHOENIX FOX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fürstin Elora</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Svela17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sphere8472</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MiepStreet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">haasenpeter rex</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MetauChopf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pawelte</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dr Cal Lightman</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tyskie 66</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skywölkchen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lilien1999</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Schlabberbacke</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MG Mayo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Xambash</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hhjjjjcg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Last Arti</t>
-  </si>
-  <si>
-    <t xml:space="preserve">케포 부인</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sunny75</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cheesynator</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dragon blou</t>
-  </si>
-  <si>
-    <t xml:space="preserve">azerty57</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sultan Murat X</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Katerina77</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EXITUS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Christo30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jukata</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Z4ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LatastrophenUlli</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jimi777</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ECSI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sanya Longer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yama Arashi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mel Lyn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kpiftw</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Last Wolf Warrior</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mischel89</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pinsel20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mac1902</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bestia77</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kurdo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leijonamieli</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GaaGol</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DooYooDoo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FATUUM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Pharo 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Toby Urbex</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VxClicker</t>
-  </si>
-  <si>
-    <t xml:space="preserve">yyyyyyyvhhmll</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R2DrehZwo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rank</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Points</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Li La Linus</t>
   </si>
   <si>
     <t xml:space="preserve">MacRoM</t>
@@ -410,7 +410,7 @@
     </font>
     <font>
       <sz val="10"/>
-      <name val="Arial"/>
+      <name val="Microsoft YaHei"/>
       <family val="2"/>
     </font>
     <font>
@@ -462,12 +462,8 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -475,7 +471,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -627,40 +623,40 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="0" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="0" t="n">
+      <c r="C2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1" t="n">
         <v>35</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C3" s="0" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3" s="0" t="n">
+      <c r="C3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="1" t="n">
         <v>45</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="0" t="s">
-        <v>1</v>
-      </c>
-      <c r="D5" s="0" t="n">
+      <c r="C5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D5" s="1" t="n">
         <v>40</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C6" s="0" t="s">
-        <v>2</v>
-      </c>
-      <c r="D6" s="0" t="n">
+      <c r="C6" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" s="1" t="n">
         <v>55</v>
       </c>
     </row>
@@ -677,7 +673,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="true">
+  <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G101"/>
@@ -687,41 +683,41 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="10.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="5.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="5.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10.38"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="1" t="n">
-        <v>137486786</v>
+      <c r="C2" s="0" t="n">
+        <v>144844997</v>
       </c>
       <c r="D2" s="1" t="str">
         <f aca="false">VLOOKUP(B2,TS!$B$2:$C$105,2,0)</f>
@@ -735,15 +731,15 @@
         <v>N</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1" t="s">
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="1" t="n">
-        <v>133705473</v>
+      <c r="C3" s="0" t="n">
+        <v>141098953</v>
       </c>
       <c r="D3" s="1" t="str">
         <f aca="false">VLOOKUP(B3,TS!$B$2:$C$105,2,0)</f>
@@ -757,15 +753,15 @@
         <v>N</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="n">
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="1" t="n">
-        <v>127073712</v>
+      <c r="C4" s="0" t="n">
+        <v>140324280</v>
       </c>
       <c r="D4" s="1" t="str">
         <f aca="false">VLOOKUP(B4,TS!$B$2:$C$105,2,0)</f>
@@ -779,15 +775,15 @@
         <v>N</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="n">
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="0" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="1" t="n">
-        <v>118975413</v>
+      <c r="C5" s="0" t="n">
+        <v>135785580</v>
       </c>
       <c r="D5" s="1" t="str">
         <f aca="false">VLOOKUP(B5,TS!$B$2:$C$105,2,0)</f>
@@ -801,15 +797,15 @@
         <v>N</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="n">
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="1" t="n">
-        <v>100503630</v>
+      <c r="C6" s="0" t="n">
+        <v>109328669</v>
       </c>
       <c r="D6" s="1" t="str">
         <f aca="false">VLOOKUP(B6,TS!$B$2:$C$105,2,0)</f>
@@ -823,59 +819,59 @@
         <v>N</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="n">
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="1" t="n">
-        <v>99128513</v>
+      <c r="C7" s="0" t="n">
+        <v>107073273</v>
       </c>
       <c r="D7" s="1" t="str">
         <f aca="false">VLOOKUP(B7,TS!$B$2:$C$105,2,0)</f>
-        <v>R4</v>
+        <v>R3</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="F7" s="1" t="str">
         <f aca="false">IF(D7&lt;&gt;E7,"Y","N")</f>
         <v>N</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="n">
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" s="1" t="n">
-        <v>96718147</v>
+        <v>17</v>
+      </c>
+      <c r="C8" s="0" t="n">
+        <v>102240483</v>
       </c>
       <c r="D8" s="1" t="str">
         <f aca="false">VLOOKUP(B8,TS!$B$2:$C$105,2,0)</f>
-        <v>R3</v>
+        <v>R4</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="F8" s="1" t="str">
         <f aca="false">IF(D8&lt;&gt;E8,"Y","N")</f>
         <v>N</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="n">
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="1" t="n">
-        <v>92070242</v>
+      <c r="C9" s="0" t="n">
+        <v>101377643</v>
       </c>
       <c r="D9" s="1" t="str">
         <f aca="false">VLOOKUP(B9,TS!$B$2:$C$105,2,0)</f>
@@ -889,15 +885,15 @@
         <v>N</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="n">
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="1" t="n">
-        <v>85880108</v>
+      <c r="C10" s="0" t="n">
+        <v>89534723</v>
       </c>
       <c r="D10" s="1" t="str">
         <f aca="false">VLOOKUP(B10,TS!$B$2:$C$105,2,0)</f>
@@ -911,81 +907,81 @@
         <v>N</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="n">
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="n">
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="1" t="n">
-        <v>81697058</v>
+      <c r="C11" s="0" t="n">
+        <v>87559780</v>
       </c>
       <c r="D11" s="1" t="str">
         <f aca="false">VLOOKUP(B11,TS!$B$2:$C$105,2,0)</f>
-        <v>R4</v>
+        <v>R3</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="F11" s="1" t="str">
         <f aca="false">IF(D11&lt;&gt;E11,"Y","N")</f>
         <v>N</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="n">
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="0" t="s">
         <v>22</v>
       </c>
-      <c r="C12" s="1" t="n">
-        <v>78710248</v>
+      <c r="C12" s="0" t="n">
+        <v>87445241</v>
       </c>
       <c r="D12" s="1" t="str">
         <f aca="false">VLOOKUP(B12,TS!$B$2:$C$105,2,0)</f>
-        <v>R3</v>
+        <v>R4</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="F12" s="1" t="str">
         <f aca="false">IF(D12&lt;&gt;E12,"Y","N")</f>
         <v>N</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1" t="n">
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="C13" s="1" t="n">
-        <v>78142688</v>
+      <c r="C13" s="0" t="n">
+        <v>81363920</v>
       </c>
       <c r="D13" s="1" t="str">
         <f aca="false">VLOOKUP(B13,TS!$B$2:$C$105,2,0)</f>
-        <v>R3</v>
+        <v>R4</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="F13" s="1" t="str">
         <f aca="false">IF(D13&lt;&gt;E13,"Y","N")</f>
         <v>N</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="1" t="n">
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="0" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="1" t="n">
-        <v>77351496</v>
+      <c r="C14" s="0" t="n">
+        <v>80852397</v>
       </c>
       <c r="D14" s="1" t="str">
         <f aca="false">VLOOKUP(B14,TS!$B$2:$C$105,2,0)</f>
@@ -999,15 +995,15 @@
         <v>N</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="1" t="n">
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="1" t="n">
-        <v>77251522</v>
+      <c r="C15" s="0" t="n">
+        <v>80293938</v>
       </c>
       <c r="D15" s="1" t="str">
         <f aca="false">VLOOKUP(B15,TS!$B$2:$C$105,2,0)</f>
@@ -1021,15 +1017,15 @@
         <v>N</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="1" t="n">
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="1" t="n">
-        <v>75233724</v>
+      <c r="C16" s="0" t="n">
+        <v>79747746</v>
       </c>
       <c r="D16" s="1" t="str">
         <f aca="false">VLOOKUP(B16,TS!$B$2:$C$105,2,0)</f>
@@ -1043,37 +1039,37 @@
         <v>N</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="1" t="n">
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="0" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="C17" s="1" t="n">
-        <v>74047701</v>
+      <c r="C17" s="0" t="n">
+        <v>79664016</v>
       </c>
       <c r="D17" s="1" t="str">
         <f aca="false">VLOOKUP(B17,TS!$B$2:$C$105,2,0)</f>
-        <v>R4</v>
+        <v>R3</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="F17" s="1" t="str">
         <f aca="false">IF(D17&lt;&gt;E17,"Y","N")</f>
         <v>N</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1" t="n">
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="C18" s="1" t="n">
-        <v>73384628</v>
+      <c r="C18" s="0" t="n">
+        <v>79577656</v>
       </c>
       <c r="D18" s="1" t="str">
         <f aca="false">VLOOKUP(B18,TS!$B$2:$C$105,2,0)</f>
@@ -1087,22 +1083,22 @@
         <v>N</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="1" t="n">
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="0" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="C19" s="1" t="n">
-        <v>73168347</v>
+      <c r="C19" s="0" t="n">
+        <v>78049804</v>
       </c>
       <c r="D19" s="1" t="str">
         <f aca="false">VLOOKUP(B19,TS!$B$2:$C$105,2,0)</f>
         <v>R4</v>
       </c>
-      <c r="E19" s="3" t="s">
-        <v>17</v>
+      <c r="E19" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="F19" s="1" t="str">
         <f aca="false">IF(D19&lt;&gt;E19,"Y","N")</f>
@@ -1110,43 +1106,43 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="1" t="n">
+      <c r="A20" s="0" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="0" t="s">
         <v>30</v>
       </c>
-      <c r="C20" s="1" t="n">
-        <v>72218502</v>
+      <c r="C20" s="0" t="n">
+        <v>76843204</v>
       </c>
       <c r="D20" s="1" t="str">
         <f aca="false">VLOOKUP(B20,TS!$B$2:$C$105,2,0)</f>
-        <v>R1</v>
+        <v>R4</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="F20" s="1" t="str">
         <f aca="false">IF(D20&lt;&gt;E20,"Y","N")</f>
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="1" t="n">
+        <v>N</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="0" t="s">
         <v>31</v>
       </c>
-      <c r="C21" s="1" t="n">
-        <v>70745578</v>
+      <c r="C21" s="0" t="n">
+        <v>76694576</v>
       </c>
       <c r="D21" s="1" t="str">
         <f aca="false">VLOOKUP(B21,TS!$B$2:$C$105,2,0)</f>
-        <v>R3</v>
+        <v>R4</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="F21" s="1" t="str">
         <f aca="false">IF(D21&lt;&gt;E21,"Y","N")</f>
@@ -1154,80 +1150,80 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="1" t="n">
+      <c r="A22" s="0" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="0" t="s">
         <v>32</v>
       </c>
-      <c r="C22" s="1" t="n">
-        <v>70291445</v>
+      <c r="C22" s="0" t="n">
+        <v>76266349</v>
       </c>
       <c r="D22" s="1" t="str">
         <f aca="false">VLOOKUP(B22,TS!$B$2:$C$105,2,0)</f>
-        <v>R2</v>
+        <v>R4</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="F22" s="1" t="str">
         <f aca="false">IF(D22&lt;&gt;E22,"Y","N")</f>
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="1" t="n">
+        <v>N</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="0" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="0" t="s">
         <v>33</v>
       </c>
-      <c r="C23" s="1" t="n">
-        <v>68952906</v>
+      <c r="C23" s="0" t="n">
+        <v>76121628</v>
       </c>
       <c r="D23" s="1" t="str">
         <f aca="false">VLOOKUP(B23,TS!$B$2:$C$105,2,0)</f>
-        <v>R4</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>17</v>
+        <v>R3</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>2</v>
       </c>
       <c r="F23" s="1" t="str">
         <f aca="false">IF(D23&lt;&gt;E23,"Y","N")</f>
         <v>N</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="1" t="n">
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="0" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" s="0" t="s">
         <v>34</v>
       </c>
-      <c r="C24" s="1" t="n">
-        <v>68453205</v>
+      <c r="C24" s="0" t="n">
+        <v>75140188</v>
       </c>
       <c r="D24" s="1" t="str">
         <f aca="false">VLOOKUP(B24,TS!$B$2:$C$105,2,0)</f>
-        <v>R4</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>17</v>
+        <v>R3</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>2</v>
       </c>
       <c r="F24" s="1" t="str">
         <f aca="false">IF(D24&lt;&gt;E24,"Y","N")</f>
         <v>N</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="1" t="n">
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="0" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" s="0" t="s">
         <v>35</v>
       </c>
-      <c r="C25" s="1" t="n">
-        <v>68223962</v>
+      <c r="C25" s="0" t="n">
+        <v>74567150</v>
       </c>
       <c r="D25" s="1" t="str">
         <f aca="false">VLOOKUP(B25,TS!$B$2:$C$105,2,0)</f>
@@ -1241,59 +1237,59 @@
         <v>N</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="1" t="n">
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="0" t="n">
         <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C26" s="1" t="n">
-        <v>68136382</v>
+      <c r="C26" s="0" t="n">
+        <v>74542017</v>
       </c>
       <c r="D26" s="1" t="str">
         <f aca="false">VLOOKUP(B26,TS!$B$2:$C$105,2,0)</f>
-        <v>R3</v>
+        <v>R2</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F26" s="1" t="str">
         <f aca="false">IF(D26&lt;&gt;E26,"Y","N")</f>
-        <v>N</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="1" t="n">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="0" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" s="0" t="s">
         <v>37</v>
       </c>
-      <c r="C27" s="1" t="n">
-        <v>67837939</v>
+      <c r="C27" s="0" t="n">
+        <v>74368502</v>
       </c>
       <c r="D27" s="1" t="str">
         <f aca="false">VLOOKUP(B27,TS!$B$2:$C$105,2,0)</f>
-        <v>R4</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>17</v>
+        <v>R1</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>2</v>
       </c>
       <c r="F27" s="1" t="str">
         <f aca="false">IF(D27&lt;&gt;E27,"Y","N")</f>
-        <v>N</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="1" t="n">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" s="0" t="s">
         <v>38</v>
       </c>
-      <c r="C28" s="1" t="n">
-        <v>67240490</v>
+      <c r="C28" s="0" t="n">
+        <v>74239148</v>
       </c>
       <c r="D28" s="1" t="str">
         <f aca="false">VLOOKUP(B28,TS!$B$2:$C$105,2,0)</f>
@@ -1307,37 +1303,37 @@
         <v>N</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="1" t="n">
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="0" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B29" s="0" t="s">
         <v>39</v>
       </c>
-      <c r="C29" s="1" t="n">
-        <v>66719174</v>
+      <c r="C29" s="0" t="n">
+        <v>71645660</v>
       </c>
       <c r="D29" s="1" t="str">
         <f aca="false">VLOOKUP(B29,TS!$B$2:$C$105,2,0)</f>
-        <v>R5</v>
+        <v>R3</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="F29" s="1" t="str">
         <f aca="false">IF(D29&lt;&gt;E29,"Y","N")</f>
         <v>N</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="1" t="n">
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0" t="n">
         <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C30" s="1" t="n">
-        <v>66419711</v>
+        <v>40</v>
+      </c>
+      <c r="C30" s="0" t="n">
+        <v>70998007</v>
       </c>
       <c r="D30" s="1" t="str">
         <f aca="false">VLOOKUP(B30,TS!$B$2:$C$105,2,0)</f>
@@ -1351,15 +1347,15 @@
         <v>N</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="1" t="n">
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="0" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C31" s="1" t="n">
-        <v>65783439</v>
+      <c r="B31" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="C31" s="0" t="n">
+        <v>70522711</v>
       </c>
       <c r="D31" s="1" t="str">
         <f aca="false">VLOOKUP(B31,TS!$B$2:$C$105,2,0)</f>
@@ -1373,15 +1369,15 @@
         <v>N</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="1" t="n">
+    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="0" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C32" s="1" t="n">
-        <v>65749582</v>
+      <c r="B32" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="C32" s="0" t="n">
+        <v>70403462</v>
       </c>
       <c r="D32" s="1" t="str">
         <f aca="false">VLOOKUP(B32,TS!$B$2:$C$105,2,0)</f>
@@ -1395,22 +1391,22 @@
         <v>N</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="1" t="n">
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="0" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C33" s="1" t="n">
-        <v>65416089</v>
+      <c r="B33" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="C33" s="0" t="n">
+        <v>69402141</v>
       </c>
       <c r="D33" s="1" t="str">
         <f aca="false">VLOOKUP(B33,TS!$B$2:$C$105,2,0)</f>
-        <v>R3</v>
+        <v>R5</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>2</v>
+        <v>44</v>
       </c>
       <c r="F33" s="1" t="str">
         <f aca="false">IF(D33&lt;&gt;E33,"Y","N")</f>
@@ -1418,36 +1414,36 @@
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="1" t="n">
+      <c r="A34" s="0" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" s="0" t="s">
         <v>45</v>
       </c>
-      <c r="C34" s="1" t="n">
-        <v>65014039</v>
+      <c r="C34" s="0" t="n">
+        <v>68434611</v>
       </c>
       <c r="D34" s="1" t="str">
         <f aca="false">VLOOKUP(B34,TS!$B$2:$C$105,2,0)</f>
-        <v>R2</v>
+        <v>R3</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F34" s="1" t="str">
         <f aca="false">IF(D34&lt;&gt;E34,"Y","N")</f>
-        <v>Y</v>
+        <v>N</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="1" t="n">
+      <c r="A35" s="0" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B35" s="0" t="s">
         <v>46</v>
       </c>
-      <c r="C35" s="1" t="n">
-        <v>63387789</v>
+      <c r="C35" s="0" t="n">
+        <v>68394289</v>
       </c>
       <c r="D35" s="1" t="str">
         <f aca="false">VLOOKUP(B35,TS!$B$2:$C$105,2,0)</f>
@@ -1461,19 +1457,19 @@
         <v>Y</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="1" t="n">
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="0" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" s="0" t="s">
         <v>47</v>
       </c>
-      <c r="C36" s="1" t="n">
-        <v>62331672</v>
+      <c r="C36" s="0" t="n">
+        <v>67428948</v>
       </c>
       <c r="D36" s="1" t="str">
         <f aca="false">VLOOKUP(B36,TS!$B$2:$C$105,2,0)</f>
-        <v>R2</v>
+        <v>R3</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>2</v>
@@ -1483,37 +1479,37 @@
       </c>
       <c r="G36" s="1"/>
     </row>
-    <row r="37" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="1" t="n">
+    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="0" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="B37" s="0" t="s">
         <v>49</v>
       </c>
-      <c r="C37" s="1" t="n">
-        <v>61182157</v>
+      <c r="C37" s="0" t="n">
+        <v>66597709</v>
       </c>
       <c r="D37" s="1" t="str">
         <f aca="false">VLOOKUP(B37,TS!$B$2:$C$105,2,0)</f>
-        <v>R3</v>
+        <v>R2</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F37" s="1" t="str">
         <f aca="false">IF(D37&lt;&gt;E37,"Y","N")</f>
-        <v>N</v>
+        <v>Y</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="1" t="n">
+      <c r="A38" s="0" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B38" s="0" t="s">
         <v>50</v>
       </c>
-      <c r="C38" s="1" t="n">
-        <v>60992085</v>
+      <c r="C38" s="0" t="n">
+        <v>65904860</v>
       </c>
       <c r="D38" s="1" t="str">
         <f aca="false">VLOOKUP(B38,TS!$B$2:$C$105,2,0)</f>
@@ -1527,22 +1523,22 @@
         <v>Y</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="1" t="n">
+    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="0" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B39" s="0" t="s">
         <v>51</v>
       </c>
-      <c r="C39" s="1" t="n">
-        <v>59977293</v>
+      <c r="C39" s="0" t="n">
+        <v>63961403</v>
       </c>
       <c r="D39" s="1" t="str">
         <f aca="false">VLOOKUP(B39,TS!$B$2:$C$105,2,0)</f>
-        <v>R3</v>
+        <v>R4</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="F39" s="1" t="str">
         <f aca="false">IF(D39&lt;&gt;E39,"Y","N")</f>
@@ -1550,14 +1546,14 @@
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="1" t="n">
+      <c r="A40" s="0" t="n">
         <v>39</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="B40" s="0" t="s">
         <v>52</v>
       </c>
-      <c r="C40" s="1" t="n">
-        <v>59618728</v>
+      <c r="C40" s="0" t="n">
+        <v>63340752</v>
       </c>
       <c r="D40" s="1" t="str">
         <f aca="false">VLOOKUP(B40,TS!$B$2:$C$105,2,0)</f>
@@ -1571,15 +1567,15 @@
         <v>Y</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="1" t="n">
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="0" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="1" t="s">
+      <c r="B41" s="0" t="s">
         <v>53</v>
       </c>
-      <c r="C41" s="1" t="n">
-        <v>58804227</v>
+      <c r="C41" s="0" t="n">
+        <v>63196589</v>
       </c>
       <c r="D41" s="1" t="str">
         <f aca="false">VLOOKUP(B41,TS!$B$2:$C$105,2,0)</f>
@@ -1593,15 +1589,15 @@
         <v>N</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="1" t="n">
+    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="0" t="n">
         <v>41</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="B42" s="0" t="s">
         <v>54</v>
       </c>
-      <c r="C42" s="1" t="n">
-        <v>57594915</v>
+      <c r="C42" s="0" t="n">
+        <v>62487102</v>
       </c>
       <c r="D42" s="1" t="str">
         <f aca="false">VLOOKUP(B42,TS!$B$2:$C$105,2,0)</f>
@@ -1615,59 +1611,59 @@
         <v>N</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="1" t="n">
+    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="0" t="n">
         <v>42</v>
       </c>
-      <c r="B43" s="1" t="s">
+      <c r="B43" s="0" t="s">
         <v>55</v>
       </c>
-      <c r="C43" s="1" t="n">
-        <v>57339470</v>
+      <c r="C43" s="0" t="n">
+        <v>62212603</v>
       </c>
       <c r="D43" s="1" t="str">
         <f aca="false">VLOOKUP(B43,TS!$B$2:$C$105,2,0)</f>
-        <v>R3</v>
+        <v>R2</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F43" s="1" t="str">
         <f aca="false">IF(D43&lt;&gt;E43,"Y","N")</f>
-        <v>N</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="1" t="n">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="0" t="n">
         <v>43</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="B44" s="0" t="s">
         <v>56</v>
       </c>
-      <c r="C44" s="1" t="n">
-        <v>57152199</v>
+      <c r="C44" s="0" t="n">
+        <v>52461027</v>
       </c>
       <c r="D44" s="1" t="str">
         <f aca="false">VLOOKUP(B44,TS!$B$2:$C$105,2,0)</f>
-        <v>R3</v>
+        <v>R2</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F44" s="1" t="str">
         <f aca="false">IF(D44&lt;&gt;E44,"Y","N")</f>
-        <v>N</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="1" t="n">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="0" t="n">
         <v>44</v>
       </c>
-      <c r="B45" s="1" t="s">
+      <c r="B45" s="0" t="s">
         <v>57</v>
       </c>
-      <c r="C45" s="1" t="n">
-        <v>57053478</v>
+      <c r="C45" s="0" t="n">
+        <v>60889716</v>
       </c>
       <c r="D45" s="1" t="str">
         <f aca="false">VLOOKUP(B45,TS!$B$2:$C$105,2,0)</f>
@@ -1681,15 +1677,15 @@
         <v>N</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="1" t="n">
+    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="0" t="n">
         <v>45</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="B46" s="0" t="s">
         <v>58</v>
       </c>
-      <c r="C46" s="1" t="n">
-        <v>56961855</v>
+      <c r="C46" s="0" t="n">
+        <v>60104199</v>
       </c>
       <c r="D46" s="1" t="str">
         <f aca="false">VLOOKUP(B46,TS!$B$2:$C$105,2,0)</f>
@@ -1703,15 +1699,15 @@
         <v>N</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="1" t="n">
+    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="0" t="n">
         <v>46</v>
       </c>
-      <c r="B47" s="1" t="s">
+      <c r="B47" s="0" t="s">
         <v>59</v>
       </c>
-      <c r="C47" s="1" t="n">
-        <v>56892881</v>
+      <c r="C47" s="0" t="n">
+        <v>59897978</v>
       </c>
       <c r="D47" s="1" t="str">
         <f aca="false">VLOOKUP(B47,TS!$B$2:$C$105,2,0)</f>
@@ -1725,37 +1721,37 @@
         <v>N</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="1" t="n">
+    <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="0" t="n">
         <v>47</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="B48" s="0" t="s">
         <v>60</v>
       </c>
-      <c r="C48" s="1" t="n">
-        <v>56714201</v>
+      <c r="C48" s="0" t="n">
+        <v>59649391</v>
       </c>
       <c r="D48" s="1" t="str">
         <f aca="false">VLOOKUP(B48,TS!$B$2:$C$105,2,0)</f>
-        <v>R4</v>
-      </c>
-      <c r="E48" s="3" t="s">
-        <v>17</v>
+        <v>R3</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>2</v>
       </c>
       <c r="F48" s="1" t="str">
         <f aca="false">IF(D48&lt;&gt;E48,"Y","N")</f>
         <v>N</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="1" t="n">
+    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="0" t="n">
         <v>48</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C49" s="1" t="n">
-        <v>55959142</v>
+      <c r="C49" s="0" t="n">
+        <v>59489470</v>
       </c>
       <c r="D49" s="1" t="str">
         <f aca="false">VLOOKUP(B49,TS!$B$2:$C$105,2,0)</f>
@@ -1769,15 +1765,15 @@
         <v>N</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="1" t="n">
+    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="0" t="n">
         <v>49</v>
       </c>
-      <c r="B50" s="1" t="s">
+      <c r="B50" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="C50" s="1" t="n">
-        <v>55914522</v>
+      <c r="C50" s="0" t="n">
+        <v>59256517</v>
       </c>
       <c r="D50" s="1" t="str">
         <f aca="false">VLOOKUP(B50,TS!$B$2:$C$105,2,0)</f>
@@ -1792,256 +1788,259 @@
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="1" t="n">
+      <c r="A51" s="0" t="n">
         <v>50</v>
       </c>
-      <c r="B51" s="1" t="s">
+      <c r="B51" s="0" t="s">
         <v>63</v>
       </c>
-      <c r="C51" s="1" t="n">
-        <v>54941797</v>
+      <c r="C51" s="0" t="n">
+        <v>58670300</v>
       </c>
       <c r="D51" s="1" t="str">
         <f aca="false">VLOOKUP(B51,TS!$B$2:$C$105,2,0)</f>
-        <v>R3</v>
+        <v>R4</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="F51" s="1" t="str">
         <f aca="false">IF(D51&lt;&gt;E51,"Y","N")</f>
-        <v>Y</v>
+        <v>N</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="1" t="n">
+      <c r="A52" s="0" t="n">
         <v>51</v>
       </c>
-      <c r="B52" s="1" t="s">
+      <c r="B52" s="0" t="s">
         <v>64</v>
       </c>
-      <c r="C52" s="1" t="n">
-        <v>54297011</v>
+      <c r="C52" s="0" t="n">
+        <v>58575395</v>
       </c>
       <c r="D52" s="1" t="str">
         <f aca="false">VLOOKUP(B52,TS!$B$2:$C$105,2,0)</f>
         <v>R1</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F52" s="1" t="str">
         <f aca="false">IF(D52&lt;&gt;E52,"Y","N")</f>
         <v>Y</v>
       </c>
+      <c r="G52" s="0" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="1" t="n">
+      <c r="A53" s="0" t="n">
         <v>52</v>
       </c>
-      <c r="B53" s="1" t="s">
+      <c r="B53" s="0" t="s">
         <v>65</v>
       </c>
-      <c r="C53" s="1" t="n">
-        <v>54281562</v>
+      <c r="C53" s="0" t="n">
+        <v>57896683</v>
       </c>
       <c r="D53" s="1" t="str">
         <f aca="false">VLOOKUP(B53,TS!$B$2:$C$105,2,0)</f>
         <v>R3</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F53" s="1" t="str">
         <f aca="false">IF(D53&lt;&gt;E53,"Y","N")</f>
-        <v>Y</v>
+        <v>N</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="1" t="n">
+      <c r="A54" s="0" t="n">
         <v>53</v>
       </c>
-      <c r="B54" s="1" t="s">
+      <c r="B54" s="0" t="s">
         <v>66</v>
       </c>
-      <c r="C54" s="1" t="n">
-        <v>52514695</v>
+      <c r="C54" s="0" t="n">
+        <v>57329285</v>
       </c>
       <c r="D54" s="1" t="str">
         <f aca="false">VLOOKUP(B54,TS!$B$2:$C$105,2,0)</f>
-        <v>R3</v>
+        <v>R4</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="F54" s="1" t="str">
         <f aca="false">IF(D54&lt;&gt;E54,"Y","N")</f>
-        <v>Y</v>
+        <v>N</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="1" t="n">
+      <c r="A55" s="0" t="n">
         <v>54</v>
       </c>
-      <c r="B55" s="1" t="s">
+      <c r="B55" s="0" t="s">
         <v>67</v>
       </c>
-      <c r="C55" s="1" t="n">
-        <v>51647419</v>
+      <c r="C55" s="0" t="n">
+        <v>57291797</v>
       </c>
       <c r="D55" s="1" t="str">
         <f aca="false">VLOOKUP(B55,TS!$B$2:$C$105,2,0)</f>
         <v>R3</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F55" s="1" t="str">
         <f aca="false">IF(D55&lt;&gt;E55,"Y","N")</f>
-        <v>Y</v>
+        <v>N</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="1" t="n">
+      <c r="A56" s="0" t="n">
         <v>55</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="B56" s="0" t="s">
         <v>68</v>
       </c>
-      <c r="C56" s="1" t="n">
-        <v>51543700</v>
+      <c r="C56" s="0" t="n">
+        <v>56859085</v>
       </c>
       <c r="D56" s="1" t="str">
         <f aca="false">VLOOKUP(B56,TS!$B$2:$C$105,2,0)</f>
         <v>R3</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F56" s="1" t="str">
         <f aca="false">IF(D56&lt;&gt;E56,"Y","N")</f>
-        <v>Y</v>
+        <v>N</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="1" t="n">
+      <c r="A57" s="0" t="n">
         <v>56</v>
       </c>
-      <c r="B57" s="1" t="s">
+      <c r="B57" s="0" t="s">
         <v>69</v>
       </c>
-      <c r="C57" s="1" t="n">
-        <v>51208865</v>
+      <c r="C57" s="0" t="n">
+        <v>56035515</v>
       </c>
       <c r="D57" s="1" t="str">
         <f aca="false">VLOOKUP(B57,TS!$B$2:$C$105,2,0)</f>
-        <v>R1</v>
+        <v>R3</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F57" s="1" t="str">
         <f aca="false">IF(D57&lt;&gt;E57,"Y","N")</f>
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="1" t="n">
+        <v>N</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="0" t="n">
         <v>57</v>
       </c>
-      <c r="B58" s="1" t="s">
+      <c r="B58" s="0" t="s">
         <v>70</v>
       </c>
-      <c r="C58" s="1" t="n">
-        <v>50423662</v>
+      <c r="C58" s="0" t="n">
+        <v>55644886</v>
       </c>
       <c r="D58" s="1" t="str">
         <f aca="false">VLOOKUP(B58,TS!$B$2:$C$105,2,0)</f>
-        <v>R4</v>
-      </c>
-      <c r="E58" s="3" t="s">
-        <v>17</v>
+        <v>R1</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>2</v>
       </c>
       <c r="F58" s="1" t="str">
         <f aca="false">IF(D58&lt;&gt;E58,"Y","N")</f>
-        <v>N</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="1" t="n">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="0" t="n">
         <v>58</v>
       </c>
-      <c r="B59" s="1" t="s">
+      <c r="B59" s="0" t="s">
         <v>71</v>
       </c>
-      <c r="C59" s="1" t="n">
-        <v>50351316</v>
+      <c r="C59" s="0" t="n">
+        <v>55072299</v>
       </c>
       <c r="D59" s="1" t="str">
         <f aca="false">VLOOKUP(B59,TS!$B$2:$C$105,2,0)</f>
-        <v>R2</v>
+        <v>R3</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F59" s="1" t="str">
         <f aca="false">IF(D59&lt;&gt;E59,"Y","N")</f>
         <v>N</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="1" t="n">
+    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="0" t="n">
         <v>59</v>
       </c>
-      <c r="B60" s="1" t="s">
+      <c r="B60" s="0" t="s">
         <v>72</v>
       </c>
-      <c r="C60" s="1" t="n">
-        <v>49849075</v>
+      <c r="C60" s="0" t="n">
+        <v>54007825</v>
       </c>
       <c r="D60" s="1" t="str">
         <f aca="false">VLOOKUP(B60,TS!$B$2:$C$105,2,0)</f>
-        <v>R4</v>
-      </c>
-      <c r="E60" s="3" t="s">
-        <v>17</v>
+        <v>R3</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="F60" s="1" t="str">
         <f aca="false">IF(D60&lt;&gt;E60,"Y","N")</f>
-        <v>N</v>
+        <v>Y</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="1" t="n">
+      <c r="A61" s="0" t="n">
         <v>60</v>
       </c>
-      <c r="B61" s="1" t="s">
+      <c r="B61" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="C61" s="1" t="n">
-        <v>49282492</v>
+      <c r="C61" s="0" t="n">
+        <v>53897808</v>
       </c>
       <c r="D61" s="1" t="str">
         <f aca="false">VLOOKUP(B61,TS!$B$2:$C$105,2,0)</f>
-        <v>R1</v>
+        <v>R2</v>
       </c>
       <c r="E61" s="1" t="s">
         <v>1</v>
       </c>
       <c r="F61" s="1" t="str">
         <f aca="false">IF(D61&lt;&gt;E61,"Y","N")</f>
-        <v>Y</v>
+        <v>N</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="1" t="n">
+      <c r="A62" s="0" t="n">
         <v>61</v>
       </c>
-      <c r="B62" s="1" t="s">
+      <c r="B62" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="C62" s="1" t="n">
-        <v>48971744</v>
+      <c r="C62" s="0" t="n">
+        <v>53325917</v>
       </c>
       <c r="D62" s="1" t="str">
         <f aca="false">VLOOKUP(B62,TS!$B$2:$C$105,2,0)</f>
@@ -2055,59 +2054,59 @@
         <v>Y</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="1" t="n">
+    <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="0" t="n">
         <v>62</v>
       </c>
-      <c r="B63" s="1" t="s">
+      <c r="B63" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="C63" s="1" t="n">
-        <v>48687647</v>
+      <c r="C63" s="0" t="n">
+        <v>52582916</v>
       </c>
       <c r="D63" s="1" t="str">
         <f aca="false">VLOOKUP(B63,TS!$B$2:$C$105,2,0)</f>
-        <v>R2</v>
+        <v>R3</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>1</v>
       </c>
       <c r="F63" s="1" t="str">
         <f aca="false">IF(D63&lt;&gt;E63,"Y","N")</f>
-        <v>N</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="1" t="n">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="0" t="n">
         <v>63</v>
       </c>
-      <c r="B64" s="1" t="s">
+      <c r="B64" s="0" t="s">
         <v>76</v>
       </c>
-      <c r="C64" s="1" t="n">
-        <v>48529362</v>
+      <c r="C64" s="0" t="n">
+        <v>52552108</v>
       </c>
       <c r="D64" s="1" t="str">
         <f aca="false">VLOOKUP(B64,TS!$B$2:$C$105,2,0)</f>
-        <v>R2</v>
+        <v>R1</v>
       </c>
       <c r="E64" s="1" t="s">
         <v>1</v>
       </c>
       <c r="F64" s="1" t="str">
         <f aca="false">IF(D64&lt;&gt;E64,"Y","N")</f>
-        <v>N</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="1" t="n">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="0" t="n">
         <v>64</v>
       </c>
-      <c r="B65" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="C65" s="1" t="n">
-        <v>48448804</v>
+      <c r="B65" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="C65" s="0" t="n">
+        <v>52461027</v>
       </c>
       <c r="D65" s="1" t="str">
         <f aca="false">VLOOKUP(B65,TS!$B$2:$C$105,2,0)</f>
@@ -2122,58 +2121,58 @@
       </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="1" t="n">
+      <c r="A66" s="0" t="n">
         <v>65</v>
       </c>
-      <c r="B66" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C66" s="1" t="n">
-        <v>48364049</v>
+      <c r="B66" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="C66" s="0" t="n">
+        <v>50510112</v>
       </c>
       <c r="D66" s="1" t="str">
         <f aca="false">VLOOKUP(B66,TS!$B$2:$C$105,2,0)</f>
-        <v>R3</v>
+        <v>R2</v>
       </c>
       <c r="E66" s="1" t="s">
         <v>1</v>
       </c>
       <c r="F66" s="1" t="str">
         <f aca="false">IF(D66&lt;&gt;E66,"Y","N")</f>
-        <v>Y</v>
+        <v>N</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="1" t="n">
+      <c r="A67" s="0" t="n">
         <v>66</v>
       </c>
-      <c r="B67" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="C67" s="1" t="n">
-        <v>47327708</v>
+      <c r="B67" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C67" s="0" t="n">
+        <v>50141804</v>
       </c>
       <c r="D67" s="1" t="str">
         <f aca="false">VLOOKUP(B67,TS!$B$2:$C$105,2,0)</f>
-        <v>R3</v>
+        <v>R2</v>
       </c>
       <c r="E67" s="1" t="s">
         <v>1</v>
       </c>
       <c r="F67" s="1" t="str">
         <f aca="false">IF(D67&lt;&gt;E67,"Y","N")</f>
-        <v>Y</v>
+        <v>N</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="1" t="n">
+      <c r="A68" s="0" t="n">
         <v>67</v>
       </c>
-      <c r="B68" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="C68" s="1" t="n">
-        <v>47276673</v>
+      <c r="B68" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="C68" s="0" t="n">
+        <v>49781583</v>
       </c>
       <c r="D68" s="1" t="str">
         <f aca="false">VLOOKUP(B68,TS!$B$2:$C$105,2,0)</f>
@@ -2188,14 +2187,14 @@
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="1" t="n">
+      <c r="A69" s="0" t="n">
         <v>68</v>
       </c>
-      <c r="B69" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C69" s="1" t="n">
-        <v>46478302</v>
+      <c r="B69" s="0" t="s">
+        <v>80</v>
+      </c>
+      <c r="C69" s="0" t="n">
+        <v>49339427</v>
       </c>
       <c r="D69" s="1" t="str">
         <f aca="false">VLOOKUP(B69,TS!$B$2:$C$105,2,0)</f>
@@ -2209,37 +2208,37 @@
         <v>Y</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="1" t="n">
+    <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="0" t="n">
         <v>69</v>
       </c>
-      <c r="B70" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C70" s="1" t="n">
-        <v>45191693</v>
+      <c r="B70" s="0" t="s">
+        <v>81</v>
+      </c>
+      <c r="C70" s="0" t="n">
+        <v>47901126</v>
       </c>
       <c r="D70" s="1" t="str">
         <f aca="false">VLOOKUP(B70,TS!$B$2:$C$105,2,0)</f>
-        <v>R2</v>
+        <v>R3</v>
       </c>
       <c r="E70" s="1" t="s">
         <v>1</v>
       </c>
       <c r="F70" s="1" t="str">
         <f aca="false">IF(D70&lt;&gt;E70,"Y","N")</f>
-        <v>N</v>
+        <v>Y</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="1" t="n">
+      <c r="A71" s="0" t="n">
         <v>70</v>
       </c>
-      <c r="B71" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="C71" s="1" t="n">
-        <v>44796126</v>
+      <c r="B71" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="C71" s="0" t="n">
+        <v>46996318</v>
       </c>
       <c r="D71" s="1" t="str">
         <f aca="false">VLOOKUP(B71,TS!$B$2:$C$105,2,0)</f>
@@ -2253,19 +2252,19 @@
         <v>Y</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="1" t="n">
+    <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="0" t="n">
         <v>71</v>
       </c>
-      <c r="B72" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="C72" s="1" t="n">
-        <v>44495693</v>
+      <c r="B72" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="C72" s="0" t="n">
+        <v>46745568</v>
       </c>
       <c r="D72" s="1" t="str">
         <f aca="false">VLOOKUP(B72,TS!$B$2:$C$105,2,0)</f>
-        <v>R3</v>
+        <v>R2</v>
       </c>
       <c r="E72" s="1" t="s">
         <v>1</v>
@@ -2276,36 +2275,36 @@
       <c r="G72" s="1"/>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="1" t="n">
+      <c r="A73" s="0" t="n">
         <v>72</v>
       </c>
-      <c r="B73" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="C73" s="1" t="n">
-        <v>43974264</v>
+      <c r="B73" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="C73" s="0" t="n">
+        <v>46325213</v>
       </c>
       <c r="D73" s="1" t="str">
         <f aca="false">VLOOKUP(B73,TS!$B$2:$C$105,2,0)</f>
-        <v>R3</v>
+        <v>R2</v>
       </c>
       <c r="E73" s="1" t="s">
         <v>1</v>
       </c>
       <c r="F73" s="1" t="str">
         <f aca="false">IF(D73&lt;&gt;E73,"Y","N")</f>
-        <v>Y</v>
+        <v>N</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="1" t="n">
+      <c r="A74" s="0" t="n">
         <v>73</v>
       </c>
-      <c r="B74" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C74" s="1" t="n">
-        <v>41756809</v>
+      <c r="B74" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="C74" s="0" t="n">
+        <v>45988139</v>
       </c>
       <c r="D74" s="1" t="str">
         <f aca="false">VLOOKUP(B74,TS!$B$2:$C$105,2,0)</f>
@@ -2320,14 +2319,14 @@
       </c>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="1" t="n">
+      <c r="A75" s="0" t="n">
         <v>74</v>
       </c>
-      <c r="B75" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C75" s="1" t="n">
-        <v>41495480</v>
+      <c r="B75" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="C75" s="0" t="n">
+        <v>45797538</v>
       </c>
       <c r="D75" s="1" t="str">
         <f aca="false">VLOOKUP(B75,TS!$B$2:$C$105,2,0)</f>
@@ -2342,18 +2341,18 @@
       </c>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="1" t="n">
+      <c r="A76" s="0" t="n">
         <v>75</v>
       </c>
-      <c r="B76" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="C76" s="1" t="n">
-        <v>41048988</v>
+      <c r="B76" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="C76" s="0" t="n">
+        <v>45471744</v>
       </c>
       <c r="D76" s="1" t="str">
         <f aca="false">VLOOKUP(B76,TS!$B$2:$C$105,2,0)</f>
-        <v>R1</v>
+        <v>R3</v>
       </c>
       <c r="E76" s="1" t="s">
         <v>1</v>
@@ -2364,18 +2363,18 @@
       </c>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="1" t="n">
+      <c r="A77" s="0" t="n">
         <v>76</v>
       </c>
-      <c r="B77" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="C77" s="1" t="n">
-        <v>40485470</v>
+      <c r="B77" s="0" t="s">
+        <v>88</v>
+      </c>
+      <c r="C77" s="0" t="n">
+        <v>45256370</v>
       </c>
       <c r="D77" s="1" t="str">
         <f aca="false">VLOOKUP(B77,TS!$B$2:$C$105,2,0)</f>
-        <v>R3</v>
+        <v>R1</v>
       </c>
       <c r="E77" s="1" t="s">
         <v>1</v>
@@ -2386,14 +2385,14 @@
       </c>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="1" t="n">
+      <c r="A78" s="0" t="n">
         <v>77</v>
       </c>
-      <c r="B78" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="C78" s="1" t="n">
-        <v>40174928</v>
+      <c r="B78" s="0" t="s">
+        <v>89</v>
+      </c>
+      <c r="C78" s="0" t="n">
+        <v>43842391</v>
       </c>
       <c r="D78" s="1" t="str">
         <f aca="false">VLOOKUP(B78,TS!$B$2:$C$105,2,0)</f>
@@ -2408,14 +2407,14 @@
       </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="1" t="n">
+      <c r="A79" s="0" t="n">
         <v>78</v>
       </c>
-      <c r="B79" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="C79" s="1" t="n">
-        <v>40138571</v>
+      <c r="B79" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="C79" s="0" t="n">
+        <v>43125220</v>
       </c>
       <c r="D79" s="1" t="str">
         <f aca="false">VLOOKUP(B79,TS!$B$2:$C$105,2,0)</f>
@@ -2430,18 +2429,18 @@
       </c>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="1" t="n">
+      <c r="A80" s="0" t="n">
         <v>79</v>
       </c>
-      <c r="B80" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C80" s="1" t="n">
-        <v>39893012</v>
+      <c r="B80" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="C80" s="0" t="n">
+        <v>42770196</v>
       </c>
       <c r="D80" s="1" t="str">
         <f aca="false">VLOOKUP(B80,TS!$B$2:$C$105,2,0)</f>
-        <v>R1</v>
+        <v>R3</v>
       </c>
       <c r="E80" s="1" t="s">
         <v>1</v>
@@ -2451,15 +2450,15 @@
         <v>Y</v>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="1" t="n">
+    <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="0" t="n">
         <v>80</v>
       </c>
-      <c r="B81" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C81" s="1" t="n">
-        <v>39875356</v>
+      <c r="B81" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="C81" s="0" t="n">
+        <v>42065371</v>
       </c>
       <c r="D81" s="1" t="str">
         <f aca="false">VLOOKUP(B81,TS!$B$2:$C$105,2,0)</f>
@@ -2473,41 +2472,41 @@
         <v>N</v>
       </c>
     </row>
-    <row r="82" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="1" t="n">
+    <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="0" t="n">
         <v>81</v>
       </c>
-      <c r="B82" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="C82" s="1" t="n">
-        <v>38821629</v>
+      <c r="B82" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="C82" s="0" t="n">
+        <v>41918803</v>
       </c>
       <c r="D82" s="1" t="str">
         <f aca="false">VLOOKUP(B82,TS!$B$2:$C$105,2,0)</f>
-        <v>R2</v>
+        <v>R3</v>
       </c>
       <c r="E82" s="1" t="s">
         <v>1</v>
       </c>
       <c r="F82" s="1" t="str">
         <f aca="false">IF(D82&lt;&gt;E82,"Y","N")</f>
-        <v>N</v>
+        <v>Y</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="1" t="n">
+      <c r="A83" s="0" t="n">
         <v>82</v>
       </c>
-      <c r="B83" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="C83" s="1" t="n">
-        <v>38153752</v>
+      <c r="B83" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="C83" s="0" t="n">
+        <v>41600387</v>
       </c>
       <c r="D83" s="1" t="str">
         <f aca="false">VLOOKUP(B83,TS!$B$2:$C$105,2,0)</f>
-        <v>R3</v>
+        <v>R1</v>
       </c>
       <c r="E83" s="1" t="s">
         <v>1</v>
@@ -2517,15 +2516,15 @@
         <v>Y</v>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="1" t="n">
+    <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="0" t="n">
         <v>83</v>
       </c>
-      <c r="B84" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="C84" s="1" t="n">
-        <v>37960623</v>
+      <c r="B84" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="C84" s="0" t="n">
+        <v>39842112</v>
       </c>
       <c r="D84" s="1" t="str">
         <f aca="false">VLOOKUP(B84,TS!$B$2:$C$105,2,0)</f>
@@ -2539,15 +2538,15 @@
         <v>N</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="1" t="n">
+    <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="0" t="n">
         <v>84</v>
       </c>
-      <c r="B85" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="C85" s="1" t="n">
-        <v>37367373</v>
+      <c r="B85" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="C85" s="0" t="n">
+        <v>39747564</v>
       </c>
       <c r="D85" s="1" t="str">
         <f aca="false">VLOOKUP(B85,TS!$B$2:$C$105,2,0)</f>
@@ -2561,15 +2560,15 @@
         <v>N</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="1" t="n">
+    <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="0" t="n">
         <v>85</v>
       </c>
-      <c r="B86" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="C86" s="1" t="n">
-        <v>36912787</v>
+      <c r="B86" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="C86" s="0" t="n">
+        <v>39676912</v>
       </c>
       <c r="D86" s="1" t="str">
         <f aca="false">VLOOKUP(B86,TS!$B$2:$C$105,2,0)</f>
@@ -2583,40 +2582,40 @@
         <v>N</v>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="1" t="n">
+    <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="0" t="n">
         <v>86</v>
       </c>
-      <c r="B87" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="C87" s="1" t="n">
-        <v>36200638</v>
+      <c r="B87" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="C87" s="0" t="n">
+        <v>38977888</v>
       </c>
       <c r="D87" s="1" t="str">
         <f aca="false">VLOOKUP(B87,TS!$B$2:$C$105,2,0)</f>
         <v>R3</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F87" s="1" t="str">
         <f aca="false">IF(D87&lt;&gt;E87,"Y","N")</f>
-        <v>N</v>
-      </c>
-      <c r="G87" s="0" t="s">
+        <v>Y</v>
+      </c>
+      <c r="G87" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="1" t="n">
+      <c r="A88" s="0" t="n">
         <v>87</v>
       </c>
-      <c r="B88" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="C88" s="1" t="n">
-        <v>35698835</v>
+      <c r="B88" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="C88" s="0" t="n">
+        <v>37901874</v>
       </c>
       <c r="D88" s="1" t="str">
         <f aca="false">VLOOKUP(B88,TS!$B$2:$C$105,2,0)</f>
@@ -2631,21 +2630,21 @@
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="1" t="n">
+      <c r="A89" s="0" t="n">
         <v>88</v>
       </c>
-      <c r="B89" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="C89" s="1" t="n">
-        <v>34731105</v>
+      <c r="B89" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="C89" s="0" t="n">
+        <v>37761450</v>
       </c>
       <c r="D89" s="1" t="str">
         <f aca="false">VLOOKUP(B89,TS!$B$2:$C$105,2,0)</f>
-        <v>R2</v>
+        <v>R3</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>102</v>
+        <v>1</v>
       </c>
       <c r="F89" s="1" t="str">
         <f aca="false">IF(D89&lt;&gt;E89,"Y","N")</f>
@@ -2653,21 +2652,21 @@
       </c>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="1" t="n">
+      <c r="A90" s="0" t="n">
         <v>89</v>
       </c>
-      <c r="B90" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="C90" s="1" t="n">
-        <v>34151064</v>
+      <c r="B90" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="C90" s="0" t="n">
+        <v>36086684</v>
       </c>
       <c r="D90" s="1" t="str">
         <f aca="false">VLOOKUP(B90,TS!$B$2:$C$105,2,0)</f>
         <v>R3</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>102</v>
+        <v>1</v>
       </c>
       <c r="F90" s="1" t="str">
         <f aca="false">IF(D90&lt;&gt;E90,"Y","N")</f>
@@ -2675,65 +2674,65 @@
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="1" t="n">
+      <c r="A91" s="0" t="n">
         <v>90</v>
       </c>
-      <c r="B91" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="C91" s="1" t="n">
-        <v>33913309</v>
+      <c r="B91" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="C91" s="0" t="n">
+        <v>36085230</v>
       </c>
       <c r="D91" s="1" t="str">
         <f aca="false">VLOOKUP(B91,TS!$B$2:$C$105,2,0)</f>
-        <v>R3</v>
+        <v>R2</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>102</v>
+        <v>1</v>
       </c>
       <c r="F91" s="1" t="str">
         <f aca="false">IF(D91&lt;&gt;E91,"Y","N")</f>
-        <v>Y</v>
+        <v>N</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="1" t="n">
+      <c r="A92" s="0" t="n">
         <v>91</v>
       </c>
-      <c r="B92" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="C92" s="1" t="n">
-        <v>32794313</v>
+      <c r="B92" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="C92" s="0" t="n">
+        <v>35187813</v>
       </c>
       <c r="D92" s="1" t="str">
         <f aca="false">VLOOKUP(B92,TS!$B$2:$C$105,2,0)</f>
         <v>R3</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>102</v>
+        <v>1</v>
       </c>
       <c r="F92" s="1" t="str">
         <f aca="false">IF(D92&lt;&gt;E92,"Y","N")</f>
         <v>Y</v>
       </c>
     </row>
-    <row r="93" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="1" t="n">
+    <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="0" t="n">
         <v>92</v>
       </c>
-      <c r="B93" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C93" s="1" t="n">
-        <v>31663743</v>
+      <c r="B93" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="C93" s="0" t="n">
+        <v>34097753</v>
       </c>
       <c r="D93" s="1" t="str">
         <f aca="false">VLOOKUP(B93,TS!$B$2:$C$105,2,0)</f>
         <v>R1</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="F93" s="1" t="str">
         <f aca="false">IF(D93&lt;&gt;E93,"Y","N")</f>
@@ -2741,43 +2740,43 @@
       </c>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="1" t="n">
+      <c r="A94" s="0" t="n">
         <v>93</v>
       </c>
-      <c r="B94" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="C94" s="1" t="n">
-        <v>28232702</v>
+      <c r="B94" s="0" t="s">
+        <v>106</v>
+      </c>
+      <c r="C94" s="0" t="n">
+        <v>31028327</v>
       </c>
       <c r="D94" s="1" t="str">
         <f aca="false">VLOOKUP(B94,TS!$B$2:$C$105,2,0)</f>
         <v>R2</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="F94" s="1" t="str">
         <f aca="false">IF(D94&lt;&gt;E94,"Y","N")</f>
         <v>Y</v>
       </c>
     </row>
-    <row r="95" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="1" t="n">
+    <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="0" t="n">
         <v>94</v>
       </c>
-      <c r="B95" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="C95" s="1" t="n">
-        <v>26376296</v>
+      <c r="B95" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="C95" s="0" t="n">
+        <v>27576296</v>
       </c>
       <c r="D95" s="1" t="str">
         <f aca="false">VLOOKUP(B95,TS!$B$2:$C$105,2,0)</f>
         <v>R1</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="F95" s="1" t="s">
         <v>48</v>
@@ -2785,42 +2784,42 @@
       <c r="G95" s="1"/>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="1" t="n">
+      <c r="A96" s="0" t="n">
         <v>95</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C96" s="1" t="n">
-        <v>24630937</v>
+        <v>108</v>
+      </c>
+      <c r="C96" s="0" t="n">
+        <v>26651251</v>
       </c>
       <c r="D96" s="1" t="str">
         <f aca="false">VLOOKUP(B96,TS!$B$2:$C$105,2,0)</f>
         <v>R2</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="F96" s="1" t="str">
         <f aca="false">IF(D96&lt;&gt;E96,"Y","N")</f>
         <v>Y</v>
       </c>
     </row>
-    <row r="97" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="1" t="n">
+    <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="0" t="n">
         <v>96</v>
       </c>
-      <c r="B97" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="C97" s="1" t="n">
+      <c r="B97" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="C97" s="0" t="n">
         <v>11684</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="F97" s="1" t="s">
         <v>48</v>
@@ -2829,28 +2828,18 @@
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="1"/>
-      <c r="F98" s="1"/>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="1"/>
-      <c r="F99" s="1"/>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="1"/>
-      <c r="F100" s="1"/>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="1"/>
-      <c r="F101" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G97">
-    <filterColumn colId="5">
-      <filters>
-        <filter val="Y"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:G97"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2877,17 +2866,17 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>113</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2895,7 +2884,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>2</v>
@@ -2909,7 +2898,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>2</v>
@@ -2923,10 +2912,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D4" s="1" t="n">
         <v>71500</v>
@@ -2937,7 +2926,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>2</v>
@@ -2951,7 +2940,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>2</v>
@@ -2979,7 +2968,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>2</v>
@@ -2993,7 +2982,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>2</v>
@@ -3007,7 +2996,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>2</v>
@@ -3021,7 +3010,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>2</v>
@@ -3035,10 +3024,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D12" s="1" t="n">
         <v>56400</v>
@@ -3049,10 +3038,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D13" s="1" t="n">
         <v>55250</v>
@@ -3063,10 +3052,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D14" s="1" t="n">
         <v>53400</v>
@@ -3077,10 +3066,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="D15" s="1" t="n">
         <v>53000</v>
@@ -3091,7 +3080,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>2</v>
@@ -3105,7 +3094,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>2</v>
@@ -3147,7 +3136,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>2</v>
@@ -3161,7 +3150,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>2</v>
@@ -3175,7 +3164,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>2</v>
@@ -3189,7 +3178,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>2</v>
@@ -3203,7 +3192,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>2</v>
@@ -3217,10 +3206,10 @@
         <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D25" s="1" t="n">
         <v>48150</v>
@@ -3231,10 +3220,10 @@
         <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D26" s="1" t="n">
         <v>47300</v>
@@ -3245,7 +3234,7 @@
         <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>2</v>
@@ -3273,7 +3262,7 @@
         <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>2</v>
@@ -3287,7 +3276,7 @@
         <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>75</v>
+        <v>56</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>1</v>
@@ -3301,7 +3290,7 @@
         <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>1</v>
@@ -3315,7 +3304,7 @@
         <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>1</v>
@@ -3329,7 +3318,7 @@
         <v>32</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>2</v>
@@ -3343,7 +3332,7 @@
         <v>33</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>2</v>
@@ -3371,7 +3360,7 @@
         <v>35</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>2</v>
@@ -3399,7 +3388,7 @@
         <v>37</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>2</v>
@@ -3427,7 +3416,7 @@
         <v>39</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>54</v>
+        <v>115</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>2</v>
@@ -3441,7 +3430,7 @@
         <v>40</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>2</v>
@@ -3455,7 +3444,7 @@
         <v>41</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>2</v>
@@ -3469,7 +3458,7 @@
         <v>42</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>2</v>
@@ -3483,7 +3472,7 @@
         <v>43</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>2</v>
@@ -3497,7 +3486,7 @@
         <v>44</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>1</v>
@@ -3511,10 +3500,10 @@
         <v>45</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D46" s="1" t="n">
         <v>42550</v>
@@ -3525,7 +3514,7 @@
         <v>46</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>2</v>
@@ -3539,7 +3528,7 @@
         <v>47</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>2</v>
@@ -3553,7 +3542,7 @@
         <v>48</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>2</v>
@@ -3567,7 +3556,7 @@
         <v>49</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>2</v>
@@ -3581,7 +3570,7 @@
         <v>50</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>2</v>
@@ -3609,10 +3598,10 @@
         <v>52</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D53" s="1" t="n">
         <v>41850</v>
@@ -3623,7 +3612,7 @@
         <v>53</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>2</v>
@@ -3637,7 +3626,7 @@
         <v>54</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>2</v>
@@ -3651,7 +3640,7 @@
         <v>55</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>1</v>
@@ -3665,7 +3654,7 @@
         <v>56</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>1</v>
@@ -3679,7 +3668,7 @@
         <v>57</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>2</v>
@@ -3693,7 +3682,7 @@
         <v>58</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>2</v>
@@ -3707,7 +3696,7 @@
         <v>59</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>2</v>
@@ -3721,10 +3710,10 @@
         <v>60</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D61" s="1" t="n">
         <v>40950</v>
@@ -3734,8 +3723,8 @@
       <c r="A62" s="1" t="n">
         <v>61</v>
       </c>
-      <c r="B62" s="4" t="s">
-        <v>77</v>
+      <c r="B62" s="3" t="s">
+        <v>78</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>1</v>
@@ -3749,7 +3738,7 @@
         <v>62</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>2</v>
@@ -3777,10 +3766,10 @@
         <v>64</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D65" s="1" t="n">
         <v>40200</v>
@@ -3791,7 +3780,7 @@
         <v>65</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C66" s="1" t="s">
         <v>2</v>
@@ -3805,10 +3794,10 @@
         <v>66</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D67" s="1" t="n">
         <v>39500</v>
@@ -3819,7 +3808,7 @@
         <v>67</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>1</v>
@@ -3833,10 +3822,10 @@
         <v>68</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D69" s="1" t="n">
         <v>39100</v>
@@ -3847,7 +3836,7 @@
         <v>69</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>1</v>
@@ -3861,7 +3850,7 @@
         <v>70</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C71" s="1" t="s">
         <v>2</v>
@@ -3889,10 +3878,10 @@
         <v>72</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D73" s="1" t="n">
         <v>38450</v>
@@ -3903,10 +3892,10 @@
         <v>73</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D74" s="1" t="n">
         <v>38400</v>
@@ -3917,7 +3906,7 @@
         <v>74</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C75" s="1" t="s">
         <v>1</v>
@@ -3931,10 +3920,10 @@
         <v>75</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D76" s="1" t="n">
         <v>38200</v>
@@ -3945,10 +3934,10 @@
         <v>76</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D77" s="1" t="n">
         <v>37750</v>
@@ -3962,7 +3951,7 @@
         <v>88</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D78" s="1" t="n">
         <v>37250</v>
@@ -3973,7 +3962,7 @@
         <v>78</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C79" s="1" t="s">
         <v>1</v>
@@ -3987,7 +3976,7 @@
         <v>79</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C80" s="1" t="s">
         <v>1</v>
@@ -4001,7 +3990,7 @@
         <v>80</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C81" s="1" t="s">
         <v>1</v>
@@ -4015,7 +4004,7 @@
         <v>81</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C82" s="1" t="s">
         <v>1</v>
@@ -4029,10 +4018,10 @@
         <v>82</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D83" s="1" t="n">
         <v>35350</v>
@@ -4043,7 +4032,7 @@
         <v>83</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C84" s="1" t="s">
         <v>2</v>
@@ -4057,7 +4046,7 @@
         <v>84</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C85" s="1" t="s">
         <v>2</v>
@@ -4071,7 +4060,7 @@
         <v>85</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C86" s="1" t="s">
         <v>1</v>
@@ -4085,7 +4074,7 @@
         <v>86</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C87" s="1" t="s">
         <v>2</v>
@@ -4113,7 +4102,7 @@
         <v>88</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C89" s="1" t="s">
         <v>2</v>
@@ -4127,7 +4116,7 @@
         <v>89</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C90" s="1" t="s">
         <v>1</v>
@@ -4141,7 +4130,7 @@
         <v>90</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C91" s="1" t="s">
         <v>1</v>
@@ -4155,7 +4144,7 @@
         <v>91</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C92" s="1" t="s">
         <v>2</v>
@@ -4169,7 +4158,7 @@
         <v>92</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C93" s="1" t="s">
         <v>1</v>
@@ -4183,7 +4172,7 @@
         <v>93</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C94" s="1" t="s">
         <v>2</v>
@@ -4197,10 +4186,10 @@
         <v>94</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D95" s="1" t="n">
         <v>20400</v>
@@ -4211,7 +4200,7 @@
         <v>95</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C96" s="1" t="s">
         <v>1</v>
@@ -4228,7 +4217,7 @@
         <v>116</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D97" s="1" t="n">
         <v>0</v>
@@ -4239,10 +4228,10 @@
         <v>97</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D98" s="1" t="n">
         <v>0</v>

</xml_diff>